<commit_message>
feat(ventas): expandir la plantilla de ventas a 72 registros y enriquecer el resumen en la interfaz
Amplía la hoja Ventas del archivo de ejemplo con 72 transacciones distribuidas en las 8 familias de productos y a lo largo de los últimos 5 días, con cantidades coherentes con las existencias para una ingesta limpia.

En la interfaz web, el resumen de ventas se enriquece calculando el ticket promedio y el promedio de unidades por venta, y la descripción del archivo descargable refleja la cobertura ampliada.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/assets/inventario_ejemplo_kardo.xlsx
+++ b/src/main/resources/static/assets/inventario_ejemplo_kardo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="745" uniqueCount="464">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="469">
   <si>
     <t xml:space="preserve">SKU</t>
   </si>
@@ -1399,10 +1399,25 @@
     <t xml:space="preserve">2026-10-20</t>
   </si>
   <si>
+    <t xml:space="preserve">BEB-VOL-010</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-10-21</t>
   </si>
   <si>
+    <t xml:space="preserve">BEB-CIF-014</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LAC-NES-011</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LIC-CRI-004</t>
+  </si>
+  <si>
     <t xml:space="preserve">2026-10-22</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BEB-SCA-009</t>
   </si>
   <si>
     <t xml:space="preserve">2026-10-23</t>
@@ -4626,10 +4641,10 @@
         <v>89</v>
       </c>
       <c r="B2" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>460</v>
+        <v>350</v>
       </c>
     </row>
     <row r="3">
@@ -4637,10 +4652,10 @@
         <v>101</v>
       </c>
       <c r="B3" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>460</v>
+        <v>350</v>
       </c>
     </row>
     <row r="4">
@@ -4648,10 +4663,10 @@
         <v>121</v>
       </c>
       <c r="B4" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="C4" t="s">
-        <v>460</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5">
@@ -4659,117 +4674,752 @@
         <v>230</v>
       </c>
       <c r="B5" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="C5" t="s">
-        <v>460</v>
+        <v>350</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>89</v>
+        <v>197</v>
       </c>
       <c r="B6" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="C6" t="s">
-        <v>461</v>
+        <v>350</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>352</v>
+        <v>11</v>
       </c>
       <c r="B7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="C7" t="s">
-        <v>461</v>
+        <v>350</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>11</v>
+        <v>25</v>
       </c>
       <c r="B8" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="C8" t="s">
-        <v>461</v>
+        <v>350</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>89</v>
+        <v>267</v>
       </c>
       <c r="B9" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>462</v>
+        <v>350</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>126</v>
+        <v>310</v>
       </c>
       <c r="B10" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C10" t="s">
-        <v>462</v>
+        <v>350</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>156</v>
+        <v>327</v>
       </c>
       <c r="B11" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="C11" t="s">
-        <v>462</v>
+        <v>350</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>236</v>
+        <v>352</v>
       </c>
       <c r="B12" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="C12" t="s">
-        <v>462</v>
+        <v>350</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>101</v>
+        <v>379</v>
       </c>
       <c r="B13" t="n">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="C13" t="s">
-        <v>463</v>
+        <v>350</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>379</v>
+        <v>156</v>
       </c>
       <c r="B14" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="C14" t="s">
-        <v>463</v>
+        <v>350</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>11</v>
+        <v>439</v>
       </c>
       <c r="B15" t="n">
         <v>4</v>
+      </c>
+      <c r="C15" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s">
+        <v>408</v>
+      </c>
+      <c r="B16" t="n">
+        <v>3</v>
+      </c>
+      <c r="C16" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B17" t="n">
+        <v>12</v>
+      </c>
+      <c r="C17" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s">
+        <v>96</v>
+      </c>
+      <c r="B18" t="n">
+        <v>5</v>
+      </c>
+      <c r="C18" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s">
+        <v>101</v>
+      </c>
+      <c r="B19" t="n">
+        <v>9</v>
+      </c>
+      <c r="C19" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s">
+        <v>461</v>
+      </c>
+      <c r="B20" t="n">
+        <v>6</v>
+      </c>
+      <c r="C20" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s">
+        <v>236</v>
+      </c>
+      <c r="B21" t="n">
+        <v>6</v>
+      </c>
+      <c r="C21" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
+        <v>210</v>
+      </c>
+      <c r="B22" t="n">
+        <v>4</v>
+      </c>
+      <c r="C22" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>11</v>
+      </c>
+      <c r="B23" t="n">
+        <v>5</v>
+      </c>
+      <c r="C23" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>51</v>
+      </c>
+      <c r="B24" t="n">
+        <v>4</v>
+      </c>
+      <c r="C24" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
+        <v>273</v>
+      </c>
+      <c r="B25" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>300</v>
+      </c>
+      <c r="B26" t="n">
+        <v>2</v>
+      </c>
+      <c r="C26" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>316</v>
+      </c>
+      <c r="B27" t="n">
+        <v>2</v>
+      </c>
+      <c r="C27" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>332</v>
+      </c>
+      <c r="B28" t="n">
+        <v>3</v>
+      </c>
+      <c r="C28" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>361</v>
+      </c>
+      <c r="B29" t="n">
+        <v>4</v>
+      </c>
+      <c r="C29" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>370</v>
+      </c>
+      <c r="B30" t="n">
+        <v>6</v>
+      </c>
+      <c r="C30" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>147</v>
+      </c>
+      <c r="B31" t="n">
+        <v>6</v>
+      </c>
+      <c r="C31" t="s">
+        <v>460</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>89</v>
+      </c>
+      <c r="B32" t="n">
+        <v>10</v>
+      </c>
+      <c r="C32" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>126</v>
+      </c>
+      <c r="B33" t="n">
+        <v>5</v>
+      </c>
+      <c r="C33" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>463</v>
+      </c>
+      <c r="B34" t="n">
+        <v>7</v>
+      </c>
+      <c r="C34" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>230</v>
+      </c>
+      <c r="B35" t="n">
+        <v>7</v>
+      </c>
+      <c r="C35" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>250</v>
+      </c>
+      <c r="B36" t="n">
+        <v>5</v>
+      </c>
+      <c r="C36" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>259</v>
+      </c>
+      <c r="B37" t="n">
+        <v>6</v>
+      </c>
+      <c r="C37" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>19</v>
+      </c>
+      <c r="B38" t="n">
+        <v>4</v>
+      </c>
+      <c r="C38" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>464</v>
+      </c>
+      <c r="B39" t="n">
+        <v>3</v>
+      </c>
+      <c r="C39" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>279</v>
+      </c>
+      <c r="B40" t="n">
+        <v>2</v>
+      </c>
+      <c r="C40" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>290</v>
+      </c>
+      <c r="B41" t="n">
+        <v>2</v>
+      </c>
+      <c r="C41" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>310</v>
+      </c>
+      <c r="B42" t="n">
+        <v>2</v>
+      </c>
+      <c r="C42" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>336</v>
+      </c>
+      <c r="B43" t="n">
+        <v>3</v>
+      </c>
+      <c r="C43" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>352</v>
+      </c>
+      <c r="B44" t="n">
+        <v>8</v>
+      </c>
+      <c r="C44" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>388</v>
+      </c>
+      <c r="B45" t="n">
+        <v>4</v>
+      </c>
+      <c r="C45" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>465</v>
+      </c>
+      <c r="B46" t="n">
+        <v>8</v>
+      </c>
+      <c r="C46" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="s">
+        <v>421</v>
+      </c>
+      <c r="B47" t="n">
+        <v>4</v>
+      </c>
+      <c r="C47" t="s">
+        <v>462</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="s">
+        <v>89</v>
+      </c>
+      <c r="B48" t="n">
+        <v>14</v>
+      </c>
+      <c r="C48" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="s">
+        <v>101</v>
+      </c>
+      <c r="B49" t="n">
+        <v>10</v>
+      </c>
+      <c r="C49" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="s">
+        <v>105</v>
+      </c>
+      <c r="B50" t="n">
+        <v>4</v>
+      </c>
+      <c r="C50" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="s">
+        <v>467</v>
+      </c>
+      <c r="B51" t="n">
+        <v>8</v>
+      </c>
+      <c r="C51" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="s">
+        <v>241</v>
+      </c>
+      <c r="B52" t="n">
+        <v>6</v>
+      </c>
+      <c r="C52" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="s">
+        <v>255</v>
+      </c>
+      <c r="B53" t="n">
+        <v>4</v>
+      </c>
+      <c r="C53" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="s">
+        <v>11</v>
+      </c>
+      <c r="B54" t="n">
+        <v>6</v>
+      </c>
+      <c r="C54" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="s">
+        <v>71</v>
+      </c>
+      <c r="B55" t="n">
+        <v>5</v>
+      </c>
+      <c r="C55" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="s">
+        <v>267</v>
+      </c>
+      <c r="B56" t="n">
+        <v>3</v>
+      </c>
+      <c r="C56" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="s">
+        <v>284</v>
+      </c>
+      <c r="B57" t="n">
+        <v>2</v>
+      </c>
+      <c r="C57" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="s">
+        <v>322</v>
+      </c>
+      <c r="B58" t="n">
+        <v>2</v>
+      </c>
+      <c r="C58" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="s">
+        <v>341</v>
+      </c>
+      <c r="B59" t="n">
+        <v>3</v>
+      </c>
+      <c r="C59" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="s">
+        <v>357</v>
+      </c>
+      <c r="B60" t="n">
+        <v>6</v>
+      </c>
+      <c r="C60" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="s">
+        <v>383</v>
+      </c>
+      <c r="B61" t="n">
+        <v>4</v>
+      </c>
+      <c r="C61" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="s">
+        <v>156</v>
+      </c>
+      <c r="B62" t="n">
+        <v>8</v>
+      </c>
+      <c r="C62" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="s">
+        <v>443</v>
+      </c>
+      <c r="B63" t="n">
+        <v>3</v>
+      </c>
+      <c r="C63" t="s">
+        <v>466</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="s">
+        <v>89</v>
+      </c>
+      <c r="B64" t="n">
+        <v>8</v>
+      </c>
+      <c r="C64" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="s">
+        <v>101</v>
+      </c>
+      <c r="B65" t="n">
+        <v>11</v>
+      </c>
+      <c r="C65" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="s">
+        <v>121</v>
+      </c>
+      <c r="B66" t="n">
+        <v>10</v>
+      </c>
+      <c r="C66" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="s">
+        <v>230</v>
+      </c>
+      <c r="B67" t="n">
+        <v>6</v>
+      </c>
+      <c r="C67" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="s">
+        <v>11</v>
+      </c>
+      <c r="B68" t="n">
+        <v>4</v>
+      </c>
+      <c r="C68" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="s">
+        <v>267</v>
+      </c>
+      <c r="B69" t="n">
+        <v>2</v>
+      </c>
+      <c r="C69" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="s">
+        <v>310</v>
+      </c>
+      <c r="B70" t="n">
+        <v>2</v>
+      </c>
+      <c r="C70" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="s">
+        <v>379</v>
+      </c>
+      <c r="B71" t="n">
+        <v>6</v>
+      </c>
+      <c r="C71" t="s">
+        <v>468</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="s">
+        <v>352</v>
+      </c>
+      <c r="B72" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="s">
+        <v>89</v>
+      </c>
+      <c r="B73" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix(demo): las ventas de ejemplo apuntaban a cinco SKU inexistentes
BEB-VOL-010, BEB-CIF-014, LAC-NES-011, LIC-CRI-004 y BEB-SCA-009 estaban en la hoja Ventas pero nunca se daban de alta en la de Inventario, asi que la carga entraba 67 de 72 y el evaluador veia cinco filas en cuarentena en su primer intento. Se sustituyen por los SKU reales a los que se parecen, de la misma familia y con stock de sobra.

El generador escribe las dos listas a mano y nada comprobaba que cuadraran. Ahora falla al generar si una venta apunta a un SKU que no existe o si la SUMA por SKU se pasa del stock -lo que agota un lote es el total de los cinco dias, no la venta mas grande-. Verificado introduciendo ambos errores a proposito.

Tamano del archivo en la pagina y captura del README, al dia.
</commit_message>
<xml_diff>
--- a/src/main/resources/static/assets/inventario_ejemplo_kardo.xlsx
+++ b/src/main/resources/static/assets/inventario_ejemplo_kardo.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="469">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="860" uniqueCount="464">
   <si>
     <t xml:space="preserve">SKU</t>
   </si>
@@ -1399,25 +1399,10 @@
     <t xml:space="preserve">2026-10-20</t>
   </si>
   <si>
-    <t xml:space="preserve">BEB-VOL-010</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-10-21</t>
   </si>
   <si>
-    <t xml:space="preserve">BEB-CIF-014</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LAC-NES-011</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LIC-CRI-004</t>
-  </si>
-  <si>
     <t xml:space="preserve">2026-10-22</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BEB-SCA-009</t>
   </si>
   <si>
     <t xml:space="preserve">2026-10-23</t>
@@ -4836,7 +4821,7 @@
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>461</v>
+        <v>134</v>
       </c>
       <c r="B20" t="n">
         <v>6</v>
@@ -4974,7 +4959,7 @@
         <v>10</v>
       </c>
       <c r="C32" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="33">
@@ -4985,18 +4970,18 @@
         <v>5</v>
       </c>
       <c r="C33" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="s">
-        <v>463</v>
+        <v>138</v>
       </c>
       <c r="B34" t="n">
         <v>7</v>
       </c>
       <c r="C34" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="35">
@@ -5007,7 +4992,7 @@
         <v>7</v>
       </c>
       <c r="C35" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="36">
@@ -5018,7 +5003,7 @@
         <v>5</v>
       </c>
       <c r="C36" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="37">
@@ -5029,7 +5014,7 @@
         <v>6</v>
       </c>
       <c r="C37" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="38">
@@ -5040,18 +5025,18 @@
         <v>4</v>
       </c>
       <c r="C38" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="s">
-        <v>464</v>
+        <v>58</v>
       </c>
       <c r="B39" t="n">
         <v>3</v>
       </c>
       <c r="C39" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="40">
@@ -5062,7 +5047,7 @@
         <v>2</v>
       </c>
       <c r="C40" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="41">
@@ -5073,7 +5058,7 @@
         <v>2</v>
       </c>
       <c r="C41" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="42">
@@ -5084,7 +5069,7 @@
         <v>2</v>
       </c>
       <c r="C42" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="43">
@@ -5095,7 +5080,7 @@
         <v>3</v>
       </c>
       <c r="C43" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="44">
@@ -5106,7 +5091,7 @@
         <v>8</v>
       </c>
       <c r="C44" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="45">
@@ -5117,18 +5102,18 @@
         <v>4</v>
       </c>
       <c r="C45" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="s">
-        <v>465</v>
+        <v>166</v>
       </c>
       <c r="B46" t="n">
         <v>8</v>
       </c>
       <c r="C46" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="47">
@@ -5139,7 +5124,7 @@
         <v>4</v>
       </c>
       <c r="C47" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
     </row>
     <row r="48">
@@ -5150,7 +5135,7 @@
         <v>14</v>
       </c>
       <c r="C48" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="49">
@@ -5161,7 +5146,7 @@
         <v>10</v>
       </c>
       <c r="C49" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="50">
@@ -5172,18 +5157,18 @@
         <v>4</v>
       </c>
       <c r="C50" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="s">
-        <v>467</v>
+        <v>130</v>
       </c>
       <c r="B51" t="n">
         <v>8</v>
       </c>
       <c r="C51" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="52">
@@ -5194,7 +5179,7 @@
         <v>6</v>
       </c>
       <c r="C52" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="53">
@@ -5205,7 +5190,7 @@
         <v>4</v>
       </c>
       <c r="C53" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="54">
@@ -5216,7 +5201,7 @@
         <v>6</v>
       </c>
       <c r="C54" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="55">
@@ -5227,7 +5212,7 @@
         <v>5</v>
       </c>
       <c r="C55" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="56">
@@ -5238,7 +5223,7 @@
         <v>3</v>
       </c>
       <c r="C56" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="57">
@@ -5249,7 +5234,7 @@
         <v>2</v>
       </c>
       <c r="C57" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="58">
@@ -5260,7 +5245,7 @@
         <v>2</v>
       </c>
       <c r="C58" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="59">
@@ -5271,7 +5256,7 @@
         <v>3</v>
       </c>
       <c r="C59" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="60">
@@ -5282,7 +5267,7 @@
         <v>6</v>
       </c>
       <c r="C60" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="61">
@@ -5293,7 +5278,7 @@
         <v>4</v>
       </c>
       <c r="C61" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="62">
@@ -5304,7 +5289,7 @@
         <v>8</v>
       </c>
       <c r="C62" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="63">
@@ -5315,7 +5300,7 @@
         <v>3</v>
       </c>
       <c r="C63" t="s">
-        <v>466</v>
+        <v>462</v>
       </c>
     </row>
     <row r="64">
@@ -5326,7 +5311,7 @@
         <v>8</v>
       </c>
       <c r="C64" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
     </row>
     <row r="65">
@@ -5337,7 +5322,7 @@
         <v>11</v>
       </c>
       <c r="C65" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
     </row>
     <row r="66">
@@ -5348,7 +5333,7 @@
         <v>10</v>
       </c>
       <c r="C66" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
     </row>
     <row r="67">
@@ -5359,7 +5344,7 @@
         <v>6</v>
       </c>
       <c r="C67" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
     </row>
     <row r="68">
@@ -5370,7 +5355,7 @@
         <v>4</v>
       </c>
       <c r="C68" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
     </row>
     <row r="69">
@@ -5381,7 +5366,7 @@
         <v>2</v>
       </c>
       <c r="C69" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
     </row>
     <row r="70">
@@ -5392,7 +5377,7 @@
         <v>2</v>
       </c>
       <c r="C70" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
     </row>
     <row r="71">
@@ -5403,7 +5388,7 @@
         <v>6</v>
       </c>
       <c r="C71" t="s">
-        <v>468</v>
+        <v>463</v>
       </c>
     </row>
     <row r="72">

</xml_diff>